<commit_message>
docs: update user stories & assignments
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -3652,12 +3652,12 @@
       <c r="J45" s="6" t="inlineStr"/>
       <c r="K45" s="6" t="inlineStr">
         <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
           <t>Lâm Phi Long</t>
-        </is>
-      </c>
-      <c r="L45" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
         </is>
       </c>
       <c r="M45" s="6" t="inlineStr">
@@ -4111,12 +4111,12 @@
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
           <t>Lâm Phi Long</t>
-        </is>
-      </c>
-      <c r="L52" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
         </is>
       </c>
       <c r="M52" s="7" t="inlineStr">
@@ -4310,10 +4310,14 @@
       </c>
       <c r="K55" s="7" t="inlineStr">
         <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="L55" s="7" t="inlineStr"/>
       <c r="M55" s="7" t="inlineStr">
         <is>
           <t>Đỗ Đăng Khoa</t>
@@ -4378,7 +4382,11 @@
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="L56" s="7" t="inlineStr"/>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
       <c r="M56" s="7" t="inlineStr">
         <is>
           <t>Đỗ Đăng Khoa</t>
@@ -4500,7 +4508,7 @@
       </c>
       <c r="L58" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Bá Tân</t>
+          <t>Trần Khải Hoàng</t>
         </is>
       </c>
       <c r="M58" s="6" t="inlineStr">
@@ -5084,14 +5092,10 @@
       </c>
       <c r="K67" s="7" t="inlineStr">
         <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="L67" s="7" t="inlineStr">
-        <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
+      <c r="L67" s="7" t="inlineStr"/>
       <c r="M67" s="7" t="inlineStr">
         <is>
           <t>Đỗ Đăng Khoa</t>
@@ -5222,7 +5226,7 @@
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>Đỗ Đăng Khoa</t>
+          <t>Nguyễn Bá Tân</t>
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr"/>
@@ -6047,7 +6051,7 @@
       <c r="J82" s="6" t="inlineStr"/>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Long</t>
+          <t>Đỗ Đăng Khoa</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr">
@@ -6311,10 +6315,14 @@
       </c>
       <c r="K86" s="7" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Long</t>
-        </is>
-      </c>
-      <c r="L86" s="7" t="inlineStr"/>
+          <t>Nguyễn Bá Tân</t>
+        </is>
+      </c>
+      <c r="L86" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
       <c r="M86" s="7" t="inlineStr">
         <is>
           <t>Đỗ Đăng Khoa</t>
@@ -6506,7 +6514,7 @@
       </c>
       <c r="K89" s="7" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Long</t>
+          <t>Đỗ Đăng Khoa</t>
         </is>
       </c>
       <c r="L89" s="7" t="inlineStr">
@@ -7243,12 +7251,12 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
           <t>Lâm Phi Long</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -7296,7 +7304,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Nguyễn Bá Tân</t>
+          <t>Trần Khải Hoàng</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -7387,7 +7395,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Nguyễn Ngọc Long</t>
+          <t>Đỗ Đăng Khoa</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -7559,24 +7567,24 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>auth, devices, devops, docs, gateway-sync, incidents, monitoring</t>
+          <t>auth, devices, devops, docs, gateway-sync, incidents</t>
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>25.6%</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -7602,20 +7610,20 @@
         </is>
       </c>
       <c r="D3" s="7" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>30.0%</t>
+          <t>26.4%</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -7676,14 +7684,14 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>auth, billing, devices, devops, trips</t>
+          <t>auth, billing, devices, trips</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>2</v>
@@ -7693,7 +7701,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>10.3%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -7719,20 +7727,20 @@
         </is>
       </c>
       <c r="D6" s="7" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>26.7%</t>
+          <t>30.3%</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -7756,10 +7764,10 @@
         <v>360</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: sync the SSOT with the module spec interview, firmware findings and field reports
Adds D-026 to D-028 and seven risk rows, ground-truth rows 19 to 23 (including the v3/v4 SOS button race and the leader's field reports on fall detection), the MF-01 order and state fixes with E02-6, E03-8 and E05-3, BR-22, the C-003 answers as 07 section 6, and backlog US-089 and US-090 with US-002 aligned to the SRS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -716,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P97"/>
+  <dimension ref="A1:P99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -977,10 +977,11 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>As a Customer (or Staff/Guide provisioned by Admin), I want to register an account with email + password, so that I can access my role's features.
-AC1: WHEN a registration request has a unique email and a password meeting policy, the system SHALL create the account and hash the password with bcrypt.
+          <t>As a Guest, I want to register a Customer account with an email verified by a one-time code, so that I can book trips and rent devices.
+AC1: WHEN a Guest submits an email and the one-time code sent to it, the system SHALL create an active Customer account whose username is the email local part, with a numeric suffix where that username is taken.
 AC2: IF the email is already registered, THEN the system SHALL reject with 409 Conflict and a field-scoped message.
-AC3: The system SHALL assign the Customer role by default; Admin/Staff/Guide accounts are provisioned by an Admin (see US-008).</t>
+AC3: WHERE a customer has no account, the system SHALL let an Operator or a Guide create the Customer account on the customer's behalf after identity verification.
+AC4: Staff accounts SHALL NOT be self-registered; they are provisioned by an Admin (see US-008). Google OAuth sign-up follows behind AUTH_GOOGLE_ENABLED.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -4077,7 +4078,7 @@
       <c r="H45" s="6" t="inlineStr"/>
       <c r="I45" s="6" t="inlineStr"/>
       <c r="J45" s="6" t="n">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
@@ -5020,88 +5021,238 @@
       <c r="P57" s="7" t="inlineStr"/>
     </row>
     <row r="58" ht="60" customHeight="1">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>E4 - Gateway &amp; Offline Sync</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>MF-02</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Staged field-event ingestion (Stages A, B and C)</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>As an Operator, I want every field event to reach the platform exactly once and in priority order, including events generated while the uplink was down, so that no SOS or position is lost.
+AC1: The system SHALL ingest events from the node uplink (Stage A), the on-device queue (Stage B) and the basecamp gateway (Stage C) through one normalizer.
+AC2: WHEN the same packet arrives more than once, the system SHALL store it once (idempotent on eventId).
+AC3: The system SHALL classify an SOS only by its text prefix, never by packet priority.</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>US-089</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>TK-97</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="inlineStr"/>
+      <c r="O58" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59" ht="60" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>E4 - Gateway &amp; Offline Sync</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>MF-02</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>On-device durable priority queue (firmware Stage B)</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>As a Guide carrying a TrekLink node out of Wi-Fi range, I want the device to hold every event it generates, in priority order and across reboots, so that an SOS raised during an outage still reaches the platform.
+AC1: The node SHALL persist queued events to flash so that they survive a reboot.
+AC2: WHEN the queue is full, the node SHALL shed the newest entry in the lowest occupied tier and SHALL never shed an SOS.
+AC3: The node SHALL publish per-tier loss counters in a queue-health report over MQTT.</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>US-090</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>TK-98</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>E4</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>Highest</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="L59" s="7" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="M59" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N59" s="7" t="inlineStr"/>
+      <c r="O59" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P59" s="7" t="inlineStr"/>
+    </row>
+    <row r="60" ht="60" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr"/>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr"/>
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>Live map/telemetry dashboard over WebSocket, automatic SOS-to-Incident creation on idempotency pass, the 5-state Incident FSM with append-only audit trail, and Staff/Guide acknowledgment-and-response workflow (MTTA/MTTR are graded RQ3 metrics).
 Primary tables/entities: incidents, incident_audit_log, device_positions (live, via WebSocket)</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>TK-5</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr"/>
-      <c r="I58" s="6" t="inlineStr"/>
-      <c r="J58" s="6" t="n">
+      <c r="H60" s="6" t="inlineStr"/>
+      <c r="I60" s="6" t="inlineStr"/>
+      <c r="J60" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="K58" s="6" t="inlineStr">
+      <c r="K60" s="6" t="inlineStr">
         <is>
           <t>Sprint 2-4 (MF-03 + MF-04)</t>
         </is>
       </c>
-      <c r="L58" s="6" t="inlineStr"/>
-      <c r="M58" s="6" t="inlineStr">
+      <c r="L60" s="6" t="inlineStr"/>
+      <c r="M60" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N58" s="6" t="inlineStr">
+      <c r="N60" s="6" t="inlineStr">
         <is>
           <t>Trần Khải Hoàng</t>
         </is>
       </c>
-      <c r="O58" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P58" s="6" t="inlineStr"/>
-    </row>
-    <row r="59" ht="60" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="O60" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61" ht="60" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr">
         <is>
           <t>MF-04</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D61" s="7" t="inlineStr">
         <is>
           <t>Device telemetry live display on map</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
+      <c r="E61" s="7" t="inlineStr">
         <is>
           <t>As Staff/Admin, I want battery and last-seen data shown on the live map markers, so that I can spot a device about to go dark before it becomes an incident.
 AC1: Markers SHALL show battery % and a relative last-seen time (e.g. "2m ago").
@@ -5109,74 +5260,74 @@
 AC3: This reuses the telemetry ingestion pipeline from US-016, no separate polling endpoint.</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
+      <c r="F61" s="7" t="inlineStr">
         <is>
           <t>US-056</t>
         </is>
       </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="G61" s="7" t="inlineStr">
         <is>
           <t>TK-64</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H61" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I59" s="7" t="inlineStr">
+      <c r="I61" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J59" s="7" t="n">
+      <c r="J61" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K59" s="7" t="inlineStr">
+      <c r="K61" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L59" s="7" t="inlineStr">
+      <c r="L61" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M59" s="7" t="inlineStr">
+      <c r="M61" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Ngọc Long</t>
         </is>
       </c>
-      <c r="N59" s="7" t="inlineStr"/>
-      <c r="O59" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P59" s="7" t="inlineStr"/>
-    </row>
-    <row r="60" ht="60" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
+      <c r="N61" s="7" t="inlineStr"/>
+      <c r="O61" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62" ht="60" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B60" s="7" t="inlineStr">
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>Append-only incident audit trail</t>
         </is>
       </c>
-      <c r="E60" s="7" t="inlineStr">
+      <c r="E62" s="7" t="inlineStr">
         <is>
           <t>As Admin, I want every incident state transition preserved permanently with actor, timestamp, and note, so that RQ3's traceability-score metric (% of transitions with complete actor+timestamp+action) can be computed directly from this data.
 AC1: Every transition from US-057 SHALL write one audit row, no update/delete endpoint SHALL exist for these rows.
@@ -5184,74 +5335,74 @@
 AC3: The audit trail SHALL be visible to Staff/Admin as a read-only timeline on the Incident detail view.</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>US-059</t>
         </is>
       </c>
-      <c r="G60" s="7" t="inlineStr">
+      <c r="G62" s="7" t="inlineStr">
         <is>
           <t>TK-67</t>
         </is>
       </c>
-      <c r="H60" s="7" t="inlineStr">
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I60" s="7" t="inlineStr">
+      <c r="I62" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J60" s="7" t="n">
+      <c r="J62" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K60" s="7" t="inlineStr">
+      <c r="K62" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L60" s="7" t="inlineStr">
+      <c r="L62" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M60" s="7" t="inlineStr">
+      <c r="M62" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N60" s="7" t="inlineStr"/>
-      <c r="O60" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P60" s="7" t="inlineStr"/>
-    </row>
-    <row r="61" ht="60" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="N62" s="7" t="inlineStr"/>
+      <c r="O62" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63" ht="60" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D63" s="7" t="inlineStr">
         <is>
           <t>Staff: acknowledge an incident</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="E63" s="7" t="inlineStr">
         <is>
           <t>As Staff, I want to acknowledge a Detected incident, so that the system records who is taking ownership and starts the response clock.
 AC1: WHEN Staff acknowledges, the system SHALL transition Detected→Acknowledged via the FSM guard (US-057).
@@ -5259,74 +5410,74 @@
 AC3: The acknowledgment action SHALL require no more than 1 step / 2 fields (button + optional note) per the time-critical UX rule (06-frontend-conventions.md §3).</t>
         </is>
       </c>
-      <c r="F61" s="7" t="inlineStr">
+      <c r="F63" s="7" t="inlineStr">
         <is>
           <t>US-060</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G63" s="7" t="inlineStr">
         <is>
           <t>TK-68</t>
         </is>
       </c>
-      <c r="H61" s="7" t="inlineStr">
+      <c r="H63" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I61" s="7" t="inlineStr">
+      <c r="I63" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J61" s="7" t="n">
+      <c r="J63" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K61" s="7" t="inlineStr">
+      <c r="K63" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L61" s="7" t="inlineStr">
+      <c r="L63" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M61" s="7" t="inlineStr">
+      <c r="M63" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N61" s="7" t="inlineStr"/>
-      <c r="O61" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P61" s="7" t="inlineStr"/>
-    </row>
-    <row r="62" ht="60" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
+      <c r="N63" s="7" t="inlineStr"/>
+      <c r="O63" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64" ht="60" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C62" s="7" t="inlineStr">
+      <c r="C64" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D62" s="7" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>Staff: update/coordinate an incident</t>
         </is>
       </c>
-      <c r="E62" s="7" t="inlineStr">
+      <c r="E64" s="7" t="inlineStr">
         <is>
           <t>As Staff, I want to transition an incident to In Progress with a coordination note, so that the response effort is documented as it happens, not reconstructed afterward.
 AC1: WHEN Staff updates status to In Progress, the system SHALL require a non-empty action note.
@@ -5334,74 +5485,74 @@
 AC3: Only Staff/Admin/the assigned Guide SHALL be authorized to update an incident's status.</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr">
+      <c r="F64" s="7" t="inlineStr">
         <is>
           <t>US-061</t>
         </is>
       </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="G64" s="7" t="inlineStr">
         <is>
           <t>TK-69</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H64" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I62" s="7" t="inlineStr">
+      <c r="I64" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J62" s="7" t="n">
+      <c r="J64" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K62" s="7" t="inlineStr">
+      <c r="K64" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L62" s="7" t="inlineStr">
+      <c r="L64" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M62" s="7" t="inlineStr">
+      <c r="M64" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N62" s="7" t="inlineStr"/>
-      <c r="O62" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P62" s="7" t="inlineStr"/>
-    </row>
-    <row r="63" ht="60" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="N64" s="7" t="inlineStr"/>
+      <c r="O64" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P64" s="7" t="inlineStr"/>
+    </row>
+    <row r="65" ht="60" customHeight="1">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D63" s="7" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>Staff: close/resolve an incident</t>
         </is>
       </c>
-      <c r="E63" s="7" t="inlineStr">
+      <c r="E65" s="7" t="inlineStr">
         <is>
           <t>As Staff, I want to transition an incident through Resolved to Closed with a resolution note, so that MTTR (a graded RQ3 metric) and the audit trail have a definite end.
 AC1: WHEN Staff resolves, the system SHALL transition In Progress→Resolved, requiring a resolution note.
@@ -5409,74 +5560,74 @@
 AC3: The Resolved timestamp SHALL be the value used for MTTR calculation (US-087).</t>
         </is>
       </c>
-      <c r="F63" s="7" t="inlineStr">
+      <c r="F65" s="7" t="inlineStr">
         <is>
           <t>US-062</t>
         </is>
       </c>
-      <c r="G63" s="7" t="inlineStr">
+      <c r="G65" s="7" t="inlineStr">
         <is>
           <t>TK-70</t>
         </is>
       </c>
-      <c r="H63" s="7" t="inlineStr">
+      <c r="H65" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I63" s="7" t="inlineStr">
+      <c r="I65" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J63" s="7" t="n">
+      <c r="J65" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K63" s="7" t="inlineStr">
+      <c r="K65" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L63" s="7" t="inlineStr">
+      <c r="L65" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M63" s="7" t="inlineStr">
+      <c r="M65" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N63" s="7" t="inlineStr"/>
-      <c r="O63" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P63" s="7" t="inlineStr"/>
-    </row>
-    <row r="64" ht="60" customHeight="1">
-      <c r="A64" s="7" t="inlineStr">
+      <c r="N65" s="7" t="inlineStr"/>
+      <c r="O65" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66" ht="60" customHeight="1">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="B66" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C66" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>Staff: manually create a non-SOS incident</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr">
+      <c r="E66" s="7" t="inlineStr">
         <is>
           <t>As Staff, I want to manually open an incident for a non-SOS emergency (e.g. a phoned-in report), so that the same tracked FSM/audit workflow applies even without a device-level SOS trigger.
 AC1: The system SHALL let Staff create an Incident directly in Detected state, optionally linked to a device/trip.
@@ -5484,74 +5635,74 @@
 AC3: The audit trail SHALL note that the incident was Staff-initiated, not device-triggered, for RQ3 baseline comparison purposes.</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
+      <c r="F66" s="7" t="inlineStr">
         <is>
           <t>US-064</t>
         </is>
       </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="G66" s="7" t="inlineStr">
         <is>
           <t>TK-72</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H66" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I64" s="7" t="inlineStr">
+      <c r="I66" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J64" s="7" t="n">
+      <c r="J66" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K64" s="7" t="inlineStr">
+      <c r="K66" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L64" s="7" t="inlineStr">
+      <c r="L66" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M64" s="7" t="inlineStr">
+      <c r="M66" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N64" s="7" t="inlineStr"/>
-      <c r="O64" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P64" s="7" t="inlineStr"/>
-    </row>
-    <row r="65" ht="60" customHeight="1">
-      <c r="A65" s="7" t="inlineStr">
+      <c r="N66" s="7" t="inlineStr"/>
+      <c r="O66" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P66" s="7" t="inlineStr"/>
+    </row>
+    <row r="67" ht="60" customHeight="1">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B65" s="7" t="inlineStr">
+      <c r="B67" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>MF-04</t>
         </is>
       </c>
-      <c r="D65" s="7" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>Gateway connectivity status indicator</t>
         </is>
       </c>
-      <c r="E65" s="7" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr">
         <is>
           <t>As Staff/Admin, I want a visible per-gateway connectivity indicator (last-seen, "syncing" vs. "stale") on the dashboard, so that a silent gateway dropout is obvious, not hidden in a tooltip (06-frontend-conventions.md §4 Pattern B).
 AC1: The indicator SHALL consume the gateway health endpoint (US-048) directly.
@@ -5559,74 +5710,74 @@
 AC3: The indicator SHALL be visible on the main dashboard, not nested behind a secondary screen.</t>
         </is>
       </c>
-      <c r="F65" s="7" t="inlineStr">
+      <c r="F67" s="7" t="inlineStr">
         <is>
           <t>US-065</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr">
+      <c r="G67" s="7" t="inlineStr">
         <is>
           <t>TK-73</t>
         </is>
       </c>
-      <c r="H65" s="7" t="inlineStr">
+      <c r="H67" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I65" s="7" t="inlineStr">
+      <c r="I67" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J65" s="7" t="n">
+      <c r="J67" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K65" s="7" t="inlineStr">
+      <c r="K67" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L65" s="7" t="inlineStr">
+      <c r="L67" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M65" s="7" t="inlineStr">
+      <c r="M67" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Ngọc Long</t>
         </is>
       </c>
-      <c r="N65" s="7" t="inlineStr"/>
-      <c r="O65" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P65" s="7" t="inlineStr"/>
-    </row>
-    <row r="66" ht="60" customHeight="1">
-      <c r="A66" s="7" t="inlineStr">
+      <c r="N67" s="7" t="inlineStr"/>
+      <c r="O67" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68" ht="60" customHeight="1">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B66" s="7" t="inlineStr">
+      <c r="B68" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C66" s="7" t="inlineStr">
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D66" s="7" t="inlineStr">
+      <c r="D68" s="7" t="inlineStr">
         <is>
           <t>Incident queue panel</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E68" s="7" t="inlineStr">
         <is>
           <t>As Staff/Admin/Guide, I want a list/filter panel of active incidents beside the map, so that an active SOS is visible without scrolling (06-frontend-conventions.md §4 Pattern B).
 AC1: The panel SHALL list incidents filterable by status and sortable by created time.
@@ -5634,74 +5785,74 @@
 AC3: Selecting an incident SHALL center the live map (US-054) on its associated device/trip.</t>
         </is>
       </c>
-      <c r="F66" s="7" t="inlineStr">
+      <c r="F68" s="7" t="inlineStr">
         <is>
           <t>US-066</t>
         </is>
       </c>
-      <c r="G66" s="7" t="inlineStr">
+      <c r="G68" s="7" t="inlineStr">
         <is>
           <t>TK-74</t>
         </is>
       </c>
-      <c r="H66" s="7" t="inlineStr">
+      <c r="H68" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I66" s="7" t="inlineStr">
+      <c r="I68" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J66" s="7" t="n">
+      <c r="J68" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K66" s="7" t="inlineStr">
+      <c r="K68" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L66" s="7" t="inlineStr">
+      <c r="L68" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M66" s="7" t="inlineStr">
+      <c r="M68" s="7" t="inlineStr">
         <is>
           <t>Trần Khải Hoàng</t>
         </is>
       </c>
-      <c r="N66" s="7" t="inlineStr"/>
-      <c r="O66" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P66" s="7" t="inlineStr"/>
-    </row>
-    <row r="67" ht="60" customHeight="1">
-      <c r="A67" s="7" t="inlineStr">
+      <c r="N68" s="7" t="inlineStr"/>
+      <c r="O68" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P68" s="7" t="inlineStr"/>
+    </row>
+    <row r="69" ht="60" customHeight="1">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B67" s="7" t="inlineStr">
+      <c r="B69" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C67" s="7" t="inlineStr">
+      <c r="C69" s="7" t="inlineStr">
         <is>
           <t>MF-04</t>
         </is>
       </c>
-      <c r="D67" s="7" t="inlineStr">
+      <c r="D69" s="7" t="inlineStr">
         <is>
           <t>WebSocket gateway (Socket.io) for live push</t>
         </is>
       </c>
-      <c r="E67" s="7" t="inlineStr">
+      <c r="E69" s="7" t="inlineStr">
         <is>
           <t>As a developer, I want one shared Socket.io gateway that all live features subscribe to, so that widgets don't each open their own connection (06-frontend-conventions.md §2).
 AC1: The system SHALL expose typed events (e.g. incident:new, device:telemetry) over a single namespace.
@@ -5709,74 +5860,74 @@
 AC3: The frontend SHALL hold this connection in one shared shared/socketClient.ts, not per-widget.</t>
         </is>
       </c>
-      <c r="F67" s="7" t="inlineStr">
+      <c r="F69" s="7" t="inlineStr">
         <is>
           <t>US-053</t>
         </is>
       </c>
-      <c r="G67" s="7" t="inlineStr">
+      <c r="G69" s="7" t="inlineStr">
         <is>
           <t>TK-61</t>
         </is>
       </c>
-      <c r="H67" s="7" t="inlineStr">
+      <c r="H69" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I67" s="7" t="inlineStr">
+      <c r="I69" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J67" s="7" t="n">
+      <c r="J69" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K67" s="7" t="inlineStr">
+      <c r="K69" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L67" s="7" t="inlineStr">
+      <c r="L69" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M67" s="7" t="inlineStr">
+      <c r="M69" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N67" s="7" t="inlineStr"/>
-      <c r="O67" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P67" s="7" t="inlineStr"/>
-    </row>
-    <row r="68" ht="60" customHeight="1">
-      <c r="A68" s="7" t="inlineStr">
+      <c r="N69" s="7" t="inlineStr"/>
+      <c r="O69" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70" ht="60" customHeight="1">
+      <c r="A70" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B68" s="7" t="inlineStr">
+      <c r="B70" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="C70" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
+      <c r="D70" s="7" t="inlineStr">
         <is>
           <t>Auto-create Incident from a valid SOS event</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr">
+      <c r="E70" s="7" t="inlineStr">
         <is>
           <t>As the system, I want to automatically create an Incident when a valid SOS event passes the idempotency check, so that no manual step stands between a firmware SOS broadcast and a tracked operational response.
 AC1: WHEN a SOS-type event passes idempotency (US-049), the system SHALL create exactly one Incident in Detected state within the same transaction.
@@ -5784,78 +5935,78 @@
 AC3: Re-delivery of the same eventId SHALL NOT create a second Incident (reuses US-049's guarantee, not a separate check).</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
+      <c r="F70" s="7" t="inlineStr">
         <is>
           <t>US-057</t>
         </is>
       </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="G70" s="7" t="inlineStr">
         <is>
           <t>TK-65</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H70" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I68" s="7" t="inlineStr">
+      <c r="I70" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J68" s="7" t="n">
+      <c r="J70" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K68" s="7" t="inlineStr">
+      <c r="K70" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L68" s="7" t="inlineStr">
+      <c r="L70" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M68" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N68" s="7" t="inlineStr">
+      <c r="M70" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N70" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Ngọc Long</t>
         </is>
       </c>
-      <c r="O68" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P68" s="7" t="inlineStr"/>
-    </row>
-    <row r="69" ht="60" customHeight="1">
-      <c r="A69" s="7" t="inlineStr">
+      <c r="O70" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71" ht="60" customHeight="1">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B69" s="7" t="inlineStr">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D69" s="7" t="inlineStr">
+      <c r="D71" s="7" t="inlineStr">
         <is>
           <t>WebSocket push notification within 2 seconds</t>
         </is>
       </c>
-      <c r="E69" s="7" t="inlineStr">
+      <c r="E71" s="7" t="inlineStr">
         <is>
           <t>As Staff/Guide, I want to be notified within 2 seconds of an Incident being created, so that response time (MTTA, a graded RQ3 metric) starts as close to real SOS trigger as possible.
 AC1: WHEN an Incident is created, the system SHALL push a notification to the assigned trip's Guide and to all online Staff/Admin within 2 seconds under normal load.
@@ -5863,74 +6014,74 @@
 AC3: This latency SHALL be measured and reported as part of US-083/US-085's RQ evaluation, not just asserted.</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr">
+      <c r="F71" s="7" t="inlineStr">
         <is>
           <t>US-058</t>
         </is>
       </c>
-      <c r="G69" s="7" t="inlineStr">
+      <c r="G71" s="7" t="inlineStr">
         <is>
           <t>TK-66</t>
         </is>
       </c>
-      <c r="H69" s="7" t="inlineStr">
+      <c r="H71" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I69" s="7" t="inlineStr">
+      <c r="I71" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J69" s="7" t="n">
+      <c r="J71" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K69" s="7" t="inlineStr">
+      <c r="K71" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L69" s="7" t="inlineStr">
+      <c r="L71" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M69" s="7" t="inlineStr">
+      <c r="M71" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N69" s="7" t="inlineStr"/>
-      <c r="O69" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P69" s="7" t="inlineStr"/>
-    </row>
-    <row r="70" ht="60" customHeight="1">
-      <c r="A70" s="7" t="inlineStr">
+      <c r="N71" s="7" t="inlineStr"/>
+      <c r="O71" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P71" s="7" t="inlineStr"/>
+    </row>
+    <row r="72" ht="60" customHeight="1">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B70" s="7" t="inlineStr">
+      <c r="B72" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr">
+      <c r="C72" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
+      <c r="D72" s="7" t="inlineStr">
         <is>
           <t>Guide: acknowledge + submit response notes</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr">
+      <c r="E72" s="7" t="inlineStr">
         <is>
           <t>As a Guide, I want to acknowledge an incident and submit response/resolution notes from the field, so that Staff has field-level context while coordinating.
 AC1: The system SHALL allow the assigned Guide to acknowledge independently of Staff's own acknowledgment, both are recorded, not merged into one flag.
@@ -5938,74 +6089,74 @@
 AC3: This flow SHALL follow the same 1-step/2-field time-critical UX rule as US-059.</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
+      <c r="F72" s="7" t="inlineStr">
         <is>
           <t>US-063</t>
         </is>
       </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="G72" s="7" t="inlineStr">
         <is>
           <t>TK-71</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
+      <c r="H72" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I70" s="7" t="inlineStr">
+      <c r="I72" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J70" s="7" t="n">
+      <c r="J72" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K70" s="7" t="inlineStr">
+      <c r="K72" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L70" s="7" t="inlineStr">
+      <c r="L72" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M70" s="7" t="inlineStr">
+      <c r="M72" s="7" t="inlineStr">
         <is>
           <t>Trần Khải Hoàng</t>
         </is>
       </c>
-      <c r="N70" s="7" t="inlineStr"/>
-      <c r="O70" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P70" s="7" t="inlineStr"/>
-    </row>
-    <row r="71" ht="60" customHeight="1">
-      <c r="A71" s="7" t="inlineStr">
+      <c r="N72" s="7" t="inlineStr"/>
+      <c r="O72" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P72" s="7" t="inlineStr"/>
+    </row>
+    <row r="73" ht="60" customHeight="1">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C73" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D73" s="7" t="inlineStr">
         <is>
           <t>Staff: distinguish and dismiss a Suspected (cadence-inferred) SOS episode</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr">
+      <c r="E73" s="7" t="inlineStr">
         <is>
           <t>As Staff, I want a cadence-inferred (Suspected) SOS episode to be visually distinct from a Confirmed one and dismissible with a lighter-weight action, so that a false-positive detection doesn't force the same evidence-heavy Resolved-to-Closed workflow as a real emergency, while a genuine SOS whose single announcing text frame was lost to RF is still surfaced instead of silently missed (gateway-sync REQ-EVT-06, the mitigation for the Critical single-unacknowledged-text-frame risk in 03-decisions-and-risk-register.md).
 AC1: WHEN the cadence-anomaly detector (gateway-sync REQ-EVT-06) raises a Suspected episode, the system SHALL create the Incident with detectionConfidence=SUSPECTED, and the map/incident-queue UI SHALL render it with a visually distinct, lower-emphasis marker/badge from a Confirmed episode (US-054, US-065's Pattern B).
@@ -6014,74 +6165,74 @@
 AC4: Dismissing a Suspected episode SHALL still write an audit row (dismissed-as-false-positive), preserving RQ3 traceability even on the non-confirmed path.</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
+      <c r="F73" s="7" t="inlineStr">
         <is>
           <t>US-088</t>
         </is>
       </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="G73" s="7" t="inlineStr">
         <is>
           <t>TK-96</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H73" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I71" s="7" t="inlineStr">
+      <c r="I73" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J71" s="7" t="n">
+      <c r="J73" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K71" s="7" t="inlineStr">
+      <c r="K73" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L71" s="7" t="inlineStr">
+      <c r="L73" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M71" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N71" s="7" t="inlineStr"/>
-      <c r="O71" s="7" t="inlineStr">
+      <c r="M73" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N73" s="7" t="inlineStr"/>
+      <c r="O73" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="P71" s="7" t="inlineStr"/>
-    </row>
-    <row r="72" ht="60" customHeight="1">
-      <c r="A72" s="7" t="inlineStr">
+      <c r="P73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74" ht="60" customHeight="1">
+      <c r="A74" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="B74" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C74" s="7" t="inlineStr">
         <is>
           <t>MF-03</t>
         </is>
       </c>
-      <c r="D72" s="7" t="inlineStr">
+      <c r="D74" s="7" t="inlineStr">
         <is>
           <t>Incident 5-state FSM engine</t>
         </is>
       </c>
-      <c r="E72" s="7" t="inlineStr">
+      <c r="E74" s="7" t="inlineStr">
         <is>
           <t>As a developer, I want an explicit transition table for Detected→Acknowledged→In Progress→Resolved→Closed, so that every incident state change is guarded and auditable, this FSM is a graded deliverable (UML State Machine diagram).
 AC1: The system SHALL reject any transition not in the allowed-transitions table, mirroring the device FSM pattern (04-architecture-conventions.md §2.1).
@@ -6089,74 +6240,74 @@
 AC3: The FSM SHALL be unit-tested for every legal transition and at least one illegal transition per state.</t>
         </is>
       </c>
-      <c r="F72" s="7" t="inlineStr">
+      <c r="F74" s="7" t="inlineStr">
         <is>
           <t>US-054</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G74" s="7" t="inlineStr">
         <is>
           <t>TK-62</t>
         </is>
       </c>
-      <c r="H72" s="7" t="inlineStr">
+      <c r="H74" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I72" s="7" t="inlineStr">
+      <c r="I74" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J72" s="7" t="n">
+      <c r="J74" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="K72" s="7" t="inlineStr">
+      <c r="K74" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L72" s="7" t="inlineStr">
+      <c r="L74" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M72" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N72" s="7" t="inlineStr"/>
-      <c r="O72" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P72" s="7" t="inlineStr"/>
-    </row>
-    <row r="73" ht="60" customHeight="1">
-      <c r="A73" s="7" t="inlineStr">
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N74" s="7" t="inlineStr"/>
+      <c r="O74" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P74" s="7" t="inlineStr"/>
+    </row>
+    <row r="75" ht="60" customHeight="1">
+      <c r="A75" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="B75" s="7" t="inlineStr">
         <is>
           <t>E5 - Real-Time Monitoring &amp; SOS Incidents</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="C75" s="7" t="inlineStr">
         <is>
           <t>MF-04</t>
         </is>
       </c>
-      <c r="D73" s="7" t="inlineStr">
+      <c r="D75" s="7" t="inlineStr">
         <is>
           <t>Live operational map (MapLibre GL + Goong Maps)</t>
         </is>
       </c>
-      <c r="E73" s="7" t="inlineStr">
+      <c r="E75" s="7" t="inlineStr">
         <is>
           <t>As Staff/Admin/Guide, I want a live map showing active trip positions, so that I have field situational awareness without polling manually.
 AC1: The map SHALL render device/trip markers colored by status per Pattern B (06-frontend-conventions.md §4).
@@ -6164,139 +6315,139 @@
 AC3: The map SHALL be the LiveMapWidget consumed by both the Staff dashboard and the Guide's own trip view (US-038).</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
+      <c r="F75" s="7" t="inlineStr">
         <is>
           <t>US-055</t>
         </is>
       </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="G75" s="7" t="inlineStr">
         <is>
           <t>TK-63</t>
         </is>
       </c>
-      <c r="H73" s="7" t="inlineStr">
+      <c r="H75" s="7" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="I73" s="7" t="inlineStr">
+      <c r="I75" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J73" s="7" t="n">
+      <c r="J75" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="K73" s="7" t="inlineStr">
+      <c r="K75" s="7" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="L73" s="7" t="inlineStr">
+      <c r="L75" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M73" s="7" t="inlineStr">
+      <c r="M75" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Ngọc Long</t>
         </is>
       </c>
-      <c r="N73" s="7" t="inlineStr">
+      <c r="N75" s="7" t="inlineStr">
         <is>
           <t>Trần Khải Hoàng</t>
         </is>
       </c>
-      <c r="O73" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P73" s="7" t="inlineStr"/>
-    </row>
-    <row r="74" ht="60" customHeight="1">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="O75" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P75" s="7" t="inlineStr"/>
+    </row>
+    <row r="76" ht="60" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr"/>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="C76" s="6" t="inlineStr"/>
+      <c r="D76" s="6" t="inlineStr">
         <is>
           <t>Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="E76" s="6" t="inlineStr">
         <is>
           <t>Rental pricing rules, automatic invoice generation, mock/sandbox payment status tracking, and usage/incident/utilization reporting for agency management.
 Primary tables/entities: pricing_rules, invoices, payments (sandbox), reports (derived views)</t>
         </is>
       </c>
-      <c r="F74" s="6" t="inlineStr">
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>TK-6</t>
         </is>
       </c>
-      <c r="H74" s="6" t="inlineStr"/>
-      <c r="I74" s="6" t="inlineStr"/>
-      <c r="J74" s="6" t="n">
+      <c r="H76" s="6" t="inlineStr"/>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="K74" s="6" t="inlineStr">
+      <c r="K76" s="6" t="inlineStr">
         <is>
           <t>Sprint 2-5 (MF-05: billing)</t>
         </is>
       </c>
-      <c r="L74" s="6" t="inlineStr"/>
-      <c r="M74" s="6" t="inlineStr">
+      <c r="L76" s="6" t="inlineStr"/>
+      <c r="M76" s="6" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N74" s="6" t="inlineStr">
+      <c r="N76" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O74" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P74" s="6" t="inlineStr"/>
-    </row>
-    <row r="75" ht="60" customHeight="1">
-      <c r="A75" s="7" t="inlineStr">
+      <c r="O76" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="60" customHeight="1">
+      <c r="A77" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B75" s="7" t="inlineStr">
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C77" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D75" s="7" t="inlineStr">
+      <c r="D77" s="7" t="inlineStr">
         <is>
           <t>View invoice &amp; payment status</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr">
+      <c r="E77" s="7" t="inlineStr">
         <is>
           <t>As a Customer/Staff, I want to view an invoice's line items and payment status, so that there's transparency on what's owed and what's been paid.
 AC1: Customers SHALL only see invoices tied to their own bookings (ownership check).
@@ -6304,74 +6455,74 @@
 AC3: This view reuses the invoice data model from US-068, no separate summarized/duplicated record.</t>
         </is>
       </c>
-      <c r="F75" s="7" t="inlineStr">
+      <c r="F77" s="7" t="inlineStr">
         <is>
           <t>US-070</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="G77" s="7" t="inlineStr">
         <is>
           <t>TK-78</t>
         </is>
       </c>
-      <c r="H75" s="7" t="inlineStr">
+      <c r="H77" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I75" s="7" t="inlineStr">
+      <c r="I77" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J75" s="7" t="n">
+      <c r="J77" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K75" s="7" t="inlineStr">
+      <c r="K77" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L75" s="7" t="inlineStr">
+      <c r="L77" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M75" s="7" t="inlineStr">
+      <c r="M77" s="7" t="inlineStr">
         <is>
           <t>Trần Khải Hoàng</t>
         </is>
       </c>
-      <c r="N75" s="7" t="inlineStr"/>
-      <c r="O75" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P75" s="7" t="inlineStr"/>
-    </row>
-    <row r="76" ht="60" customHeight="1">
-      <c r="A76" s="7" t="inlineStr">
+      <c r="N77" s="7" t="inlineStr"/>
+      <c r="O77" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P77" s="7" t="inlineStr"/>
+    </row>
+    <row r="78" ht="60" customHeight="1">
+      <c r="A78" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B76" s="7" t="inlineStr">
+      <c r="B78" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C76" s="7" t="inlineStr">
+      <c r="C78" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D76" s="7" t="inlineStr">
+      <c r="D78" s="7" t="inlineStr">
         <is>
           <t>System health &amp; audit-log report view</t>
         </is>
       </c>
-      <c r="E76" s="7" t="inlineStr">
+      <c r="E78" s="7" t="inlineStr">
         <is>
           <t>As Admin, I want a view of system health (gateway connectivity summary, audit-log volume), so that operational health is visible without querying the database directly.
 AC1: The view SHALL summarize gateway health (US-048) across all active gateways, not just one.
@@ -6379,74 +6530,74 @@
 AC3: This view is Admin-only (RBAC-gated, not visible to Staff).</t>
         </is>
       </c>
-      <c r="F76" s="7" t="inlineStr">
+      <c r="F78" s="7" t="inlineStr">
         <is>
           <t>US-073</t>
         </is>
       </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="G78" s="7" t="inlineStr">
         <is>
           <t>TK-81</t>
         </is>
       </c>
-      <c r="H76" s="7" t="inlineStr">
+      <c r="H78" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I76" s="7" t="inlineStr">
+      <c r="I78" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J76" s="7" t="n">
+      <c r="J78" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K76" s="7" t="inlineStr">
+      <c r="K78" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L76" s="7" t="inlineStr">
+      <c r="L78" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M76" s="7" t="inlineStr">
+      <c r="M78" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Ngọc Long</t>
         </is>
       </c>
-      <c r="N76" s="7" t="inlineStr"/>
-      <c r="O76" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P76" s="7" t="inlineStr"/>
-    </row>
-    <row r="77" ht="60" customHeight="1">
-      <c r="A77" s="7" t="inlineStr">
+      <c r="N78" s="7" t="inlineStr"/>
+      <c r="O78" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P78" s="7" t="inlineStr"/>
+    </row>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B77" s="7" t="inlineStr">
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C77" s="7" t="inlineStr">
+      <c r="C79" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D77" s="7" t="inlineStr">
+      <c r="D79" s="7" t="inlineStr">
         <is>
           <t>Billing dashboard widget</t>
         </is>
       </c>
-      <c r="E77" s="7" t="inlineStr">
+      <c r="E79" s="7" t="inlineStr">
         <is>
           <t>As Staff/Admin, I want a summary widget of revenue and outstanding payments, so that billing status is visible at a glance from the main dashboard.
 AC1: The widget SHALL show total revenue and total outstanding (Pending) payments for a selectable period.
@@ -6454,74 +6605,74 @@
 AC3: Clicking the widget SHALL deep-link to the filtered invoice list.</t>
         </is>
       </c>
-      <c r="F77" s="7" t="inlineStr">
+      <c r="F79" s="7" t="inlineStr">
         <is>
           <t>US-074</t>
         </is>
       </c>
-      <c r="G77" s="7" t="inlineStr">
+      <c r="G79" s="7" t="inlineStr">
         <is>
           <t>TK-82</t>
         </is>
       </c>
-      <c r="H77" s="7" t="inlineStr">
+      <c r="H79" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I77" s="7" t="inlineStr">
+      <c r="I79" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J77" s="7" t="n">
+      <c r="J79" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K77" s="7" t="inlineStr">
+      <c r="K79" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L77" s="7" t="inlineStr">
+      <c r="L79" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M77" s="7" t="inlineStr">
+      <c r="M79" s="7" t="inlineStr">
         <is>
           <t>Trần Khải Hoàng</t>
         </is>
       </c>
-      <c r="N77" s="7" t="inlineStr"/>
-      <c r="O77" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P77" s="7" t="inlineStr"/>
-    </row>
-    <row r="78" ht="60" customHeight="1">
-      <c r="A78" s="7" t="inlineStr">
+      <c r="N79" s="7" t="inlineStr"/>
+      <c r="O79" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P79" s="7" t="inlineStr"/>
+    </row>
+    <row r="80" ht="60" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B78" s="7" t="inlineStr">
+      <c r="B80" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C78" s="7" t="inlineStr">
+      <c r="C80" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D78" s="7" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>Mock/sandbox payment integration</t>
         </is>
       </c>
-      <c r="E78" s="7" t="inlineStr">
+      <c r="E80" s="7" t="inlineStr">
         <is>
           <t>As the system, I want a mock/sandbox payment flow with status tracking (Pending/Paid/Failed), so that the billing workflow is demonstrable without a production payment gateway, per the register's explicit MVP scope.
 AC1: The system SHALL mark every transaction with a sandbox:true flag per the WHERE-clause requirement in the register.
@@ -6529,74 +6680,74 @@
 AC3: This SHALL be clearly labeled as sandbox in both API responses and the UI, so it's never mistaken for a real charge.</t>
         </is>
       </c>
-      <c r="F78" s="7" t="inlineStr">
+      <c r="F80" s="7" t="inlineStr">
         <is>
           <t>US-069</t>
         </is>
       </c>
-      <c r="G78" s="7" t="inlineStr">
+      <c r="G80" s="7" t="inlineStr">
         <is>
           <t>TK-77</t>
         </is>
       </c>
-      <c r="H78" s="7" t="inlineStr">
+      <c r="H80" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I78" s="7" t="inlineStr">
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J78" s="7" t="n">
+      <c r="J80" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K78" s="7" t="inlineStr">
+      <c r="K80" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L78" s="7" t="inlineStr">
+      <c r="L80" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M78" s="7" t="inlineStr">
+      <c r="M80" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N78" s="7" t="inlineStr"/>
-      <c r="O78" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P78" s="7" t="inlineStr"/>
-    </row>
-    <row r="79" ht="60" customHeight="1">
-      <c r="A79" s="7" t="inlineStr">
+      <c r="N80" s="7" t="inlineStr"/>
+      <c r="O80" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P80" s="7" t="inlineStr"/>
+    </row>
+    <row r="81" ht="60" customHeight="1">
+      <c r="A81" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B79" s="7" t="inlineStr">
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C79" s="7" t="inlineStr">
+      <c r="C81" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D79" s="7" t="inlineStr">
+      <c r="D81" s="7" t="inlineStr">
         <is>
           <t>Usage &amp; device-utilization report</t>
         </is>
       </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="E81" s="7" t="inlineStr">
         <is>
           <t>As Admin/Staff, I want a report on rentals and device utilization, so that fleet sizing and pricing decisions have data behind them.
 AC1: The report SHALL show rental counts and per-device utilization % over a selectable date range.
@@ -6604,74 +6755,74 @@
 AC3: The report SHALL be exportable (CSV) for the SRS/documentation deliverable.</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr">
+      <c r="F81" s="7" t="inlineStr">
         <is>
           <t>US-071</t>
         </is>
       </c>
-      <c r="G79" s="7" t="inlineStr">
+      <c r="G81" s="7" t="inlineStr">
         <is>
           <t>TK-79</t>
         </is>
       </c>
-      <c r="H79" s="7" t="inlineStr">
+      <c r="H81" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I79" s="7" t="inlineStr">
+      <c r="I81" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J79" s="7" t="n">
+      <c r="J81" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K79" s="7" t="inlineStr">
+      <c r="K81" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L79" s="7" t="inlineStr">
+      <c r="L81" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M79" s="7" t="inlineStr">
+      <c r="M81" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N79" s="7" t="inlineStr"/>
-      <c r="O79" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P79" s="7" t="inlineStr"/>
-    </row>
-    <row r="80" ht="60" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
+      <c r="N81" s="7" t="inlineStr"/>
+      <c r="O81" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P81" s="7" t="inlineStr"/>
+    </row>
+    <row r="82" ht="60" customHeight="1">
+      <c r="A82" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B80" s="7" t="inlineStr">
+      <c r="B82" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="D82" s="7" t="inlineStr">
         <is>
           <t>Incident / response-performance report</t>
         </is>
       </c>
-      <c r="E80" s="7" t="inlineStr">
+      <c r="E82" s="7" t="inlineStr">
         <is>
           <t>As Admin, I want a report summarizing incident counts, MTTA, and MTTR over time, so that response-team performance is visible to management (this doubles as input to US-087's evaluation report).
 AC1: The report SHALL compute MTTA/MTTR from the incident audit trail (US-064) directly, matching the calculation used in US-087.
@@ -6679,74 +6830,74 @@
 AC3: The report SHALL be exportable (CSV).</t>
         </is>
       </c>
-      <c r="F80" s="7" t="inlineStr">
+      <c r="F82" s="7" t="inlineStr">
         <is>
           <t>US-072</t>
         </is>
       </c>
-      <c r="G80" s="7" t="inlineStr">
+      <c r="G82" s="7" t="inlineStr">
         <is>
           <t>TK-80</t>
         </is>
       </c>
-      <c r="H80" s="7" t="inlineStr">
+      <c r="H82" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I80" s="7" t="inlineStr">
+      <c r="I82" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J80" s="7" t="n">
+      <c r="J82" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K80" s="7" t="inlineStr">
+      <c r="K82" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L80" s="7" t="inlineStr">
+      <c r="L82" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M80" s="7" t="inlineStr">
+      <c r="M82" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N80" s="7" t="inlineStr"/>
-      <c r="O80" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P80" s="7" t="inlineStr"/>
-    </row>
-    <row r="81" ht="60" customHeight="1">
-      <c r="A81" s="7" t="inlineStr">
+      <c r="N82" s="7" t="inlineStr"/>
+      <c r="O82" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P82" s="7" t="inlineStr"/>
+    </row>
+    <row r="83" ht="60" customHeight="1">
+      <c r="A83" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B81" s="7" t="inlineStr">
+      <c r="B83" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C81" s="7" t="inlineStr">
+      <c r="C83" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D81" s="7" t="inlineStr">
+      <c r="D83" s="7" t="inlineStr">
         <is>
           <t>Manage rental pricing rules</t>
         </is>
       </c>
-      <c r="E81" s="7" t="inlineStr">
+      <c r="E83" s="7" t="inlineStr">
         <is>
           <t>As an Admin, I want to configure pricing rules (per device type, per day/trip, late-fee and damage-fee formulas), so that fee calculation (US-035/036) and invoicing (US-068) aren't hardcoded.
 AC1: The system SHALL let Admin define a base rate per device type and per day/trip.
@@ -6754,74 +6905,74 @@
 AC3: A pricing-rule change SHALL apply only to new agreements going forward, never retroactively to signed agreements (matches US-023's non-retroactive principle).</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr">
+      <c r="F83" s="7" t="inlineStr">
         <is>
           <t>US-067</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr">
+      <c r="G83" s="7" t="inlineStr">
         <is>
           <t>TK-75</t>
         </is>
       </c>
-      <c r="H81" s="7" t="inlineStr">
+      <c r="H83" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I81" s="7" t="inlineStr">
+      <c r="I83" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J81" s="7" t="n">
+      <c r="J83" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K81" s="7" t="inlineStr">
+      <c r="K83" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L81" s="7" t="inlineStr">
+      <c r="L83" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M81" s="7" t="inlineStr">
+      <c r="M83" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N81" s="7" t="inlineStr"/>
-      <c r="O81" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P81" s="7" t="inlineStr"/>
-    </row>
-    <row r="82" ht="60" customHeight="1">
-      <c r="A82" s="7" t="inlineStr">
+      <c r="N83" s="7" t="inlineStr"/>
+      <c r="O83" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P83" s="7" t="inlineStr"/>
+    </row>
+    <row r="84" ht="60" customHeight="1">
+      <c r="A84" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B82" s="7" t="inlineStr">
+      <c r="B84" s="7" t="inlineStr">
         <is>
           <t>E6 - Billing &amp; Reporting</t>
         </is>
       </c>
-      <c r="C82" s="7" t="inlineStr">
+      <c r="C84" s="7" t="inlineStr">
         <is>
           <t>MF-05</t>
         </is>
       </c>
-      <c r="D82" s="7" t="inlineStr">
+      <c r="D84" s="7" t="inlineStr">
         <is>
           <t>Automatic invoice generation</t>
         </is>
       </c>
-      <c r="E82" s="7" t="inlineStr">
+      <c r="E84" s="7" t="inlineStr">
         <is>
           <t>As the system, I want to generate an invoice automatically from a completed rental agreement (base charge + late fee + damage fee), so that Staff don't manually tally charges.
 AC1: WHEN check-in (US-034) completes and all fees (US-035/036) are calculated, the system SHALL generate one invoice itemizing base/late/damage charges.
@@ -6829,135 +6980,135 @@
 AC3: Invoice generation SHALL be idempotent per rental agreement (re-triggering it SHALL NOT create a duplicate invoice).</t>
         </is>
       </c>
-      <c r="F82" s="7" t="inlineStr">
+      <c r="F84" s="7" t="inlineStr">
         <is>
           <t>US-068</t>
         </is>
       </c>
-      <c r="G82" s="7" t="inlineStr">
+      <c r="G84" s="7" t="inlineStr">
         <is>
           <t>TK-76</t>
         </is>
       </c>
-      <c r="H82" s="7" t="inlineStr">
+      <c r="H84" s="7" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
       </c>
-      <c r="I82" s="7" t="inlineStr">
+      <c r="I84" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J82" s="7" t="n">
+      <c r="J84" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K82" s="7" t="inlineStr">
+      <c r="K84" s="7" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="L82" s="7" t="inlineStr">
+      <c r="L84" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M82" s="7" t="inlineStr">
+      <c r="M84" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N82" s="7" t="inlineStr"/>
-      <c r="O82" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P82" s="7" t="inlineStr"/>
-    </row>
-    <row r="83" ht="60" customHeight="1">
-      <c r="A83" s="6" t="inlineStr">
+      <c r="N84" s="7" t="inlineStr"/>
+      <c r="O84" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P84" s="7" t="inlineStr"/>
+    </row>
+    <row r="85" ht="60" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="B83" s="6" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C83" s="6" t="inlineStr"/>
-      <c r="D83" s="6" t="inlineStr">
+      <c r="C85" s="6" t="inlineStr"/>
+      <c r="D85" s="6" t="inlineStr">
         <is>
           <t>DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="E83" s="6" t="inlineStr">
+      <c r="E85" s="6" t="inlineStr">
         <is>
           <t>Docker Compose for all services, GitHub Actions CI (lint/typecheck/test/build) and CD, health-check endpoint, environment configuration matrix, deployment guide, and demo seed data.
 Primary tables/entities: n/a (infrastructure)</t>
         </is>
       </c>
-      <c r="F83" s="6" t="inlineStr">
+      <c r="F85" s="6" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="G85" s="6" t="inlineStr">
         <is>
           <t>TK-7</t>
         </is>
       </c>
-      <c r="H83" s="6" t="inlineStr"/>
-      <c r="I83" s="6" t="inlineStr"/>
-      <c r="J83" s="6" t="n">
+      <c r="H85" s="6" t="inlineStr"/>
+      <c r="I85" s="6" t="inlineStr"/>
+      <c r="J85" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="K83" s="6" t="inlineStr">
+      <c r="K85" s="6" t="inlineStr">
         <is>
           <t>Sprint 1 then ongoing (cross-cutting, not a Main Flow)</t>
         </is>
       </c>
-      <c r="L83" s="6" t="inlineStr"/>
-      <c r="M83" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N83" s="6" t="inlineStr">
+      <c r="L85" s="6" t="inlineStr"/>
+      <c r="M85" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N85" s="6" t="inlineStr">
         <is>
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="O83" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P83" s="6" t="inlineStr"/>
-    </row>
-    <row r="84" ht="60" customHeight="1">
-      <c r="A84" s="7" t="inlineStr">
+      <c r="O85" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86" ht="60" customHeight="1">
+      <c r="A86" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B84" s="7" t="inlineStr">
+      <c r="B86" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C84" s="7" t="inlineStr">
+      <c r="C86" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D84" s="7" t="inlineStr">
+      <c r="D86" s="7" t="inlineStr">
         <is>
           <t>Backend health-check endpoint</t>
         </is>
       </c>
-      <c r="E84" s="7" t="inlineStr">
+      <c r="E86" s="7" t="inlineStr">
         <is>
           <t>As Ops, I want a `/health` endpoint, so that uptime monitoring and the deployment guide have something concrete to point at.
 AC1: The endpoint SHALL report basic liveness (process up) without requiring auth.
@@ -6965,74 +7116,74 @@
 AC3: The endpoint SHALL use the standard response envelope like every other endpoint (no special-cased shape).</t>
         </is>
       </c>
-      <c r="F84" s="7" t="inlineStr">
+      <c r="F86" s="7" t="inlineStr">
         <is>
           <t>US-077</t>
         </is>
       </c>
-      <c r="G84" s="7" t="inlineStr">
+      <c r="G86" s="7" t="inlineStr">
         <is>
           <t>TK-85</t>
         </is>
       </c>
-      <c r="H84" s="7" t="inlineStr">
+      <c r="H86" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I84" s="7" t="inlineStr">
+      <c r="I86" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J84" s="7" t="n">
+      <c r="J86" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K84" s="7" t="inlineStr">
+      <c r="K86" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L84" s="7" t="inlineStr">
+      <c r="L86" s="7" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
-      <c r="M84" s="7" t="inlineStr">
+      <c r="M86" s="7" t="inlineStr">
         <is>
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="N84" s="7" t="inlineStr"/>
-      <c r="O84" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P84" s="7" t="inlineStr"/>
-    </row>
-    <row r="85" ht="60" customHeight="1">
-      <c r="A85" s="7" t="inlineStr">
+      <c r="N86" s="7" t="inlineStr"/>
+      <c r="O86" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P86" s="7" t="inlineStr"/>
+    </row>
+    <row r="87" ht="60" customHeight="1">
+      <c r="A87" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B85" s="7" t="inlineStr">
+      <c r="B87" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C85" s="7" t="inlineStr">
+      <c r="C87" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D85" s="7" t="inlineStr">
+      <c r="D87" s="7" t="inlineStr">
         <is>
           <t>Environment configuration matrix</t>
         </is>
       </c>
-      <c r="E85" s="7" t="inlineStr">
+      <c r="E87" s="7" t="inlineStr">
         <is>
           <t>As a developer, I want .env.example fully covering every variable each package actually reads, so that onboarding doesn't involve guessing missing config.
 AC1: Every env var referenced in backend/gateway/frontend source SHALL have a corresponding entry in .env.example with a comment.
@@ -7040,74 +7191,74 @@
 AC3: The README's setup section SHALL reference this file rather than duplicating the variable list inline.</t>
         </is>
       </c>
-      <c r="F85" s="7" t="inlineStr">
+      <c r="F87" s="7" t="inlineStr">
         <is>
           <t>US-079</t>
         </is>
       </c>
-      <c r="G85" s="7" t="inlineStr">
+      <c r="G87" s="7" t="inlineStr">
         <is>
           <t>TK-87</t>
         </is>
       </c>
-      <c r="H85" s="7" t="inlineStr">
+      <c r="H87" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I85" s="7" t="inlineStr">
+      <c r="I87" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J85" s="7" t="n">
+      <c r="J87" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K85" s="7" t="inlineStr">
+      <c r="K87" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L85" s="7" t="inlineStr">
+      <c r="L87" s="7" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
-      <c r="M85" s="7" t="inlineStr">
+      <c r="M87" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N85" s="7" t="inlineStr"/>
-      <c r="O85" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P85" s="7" t="inlineStr"/>
-    </row>
-    <row r="86" ht="60" customHeight="1">
-      <c r="A86" s="7" t="inlineStr">
+      <c r="N87" s="7" t="inlineStr"/>
+      <c r="O87" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P87" s="7" t="inlineStr"/>
+    </row>
+    <row r="88" ht="60" customHeight="1">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B86" s="7" t="inlineStr">
+      <c r="B88" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C86" s="7" t="inlineStr">
+      <c r="C88" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D86" s="7" t="inlineStr">
+      <c r="D88" s="7" t="inlineStr">
         <is>
           <t>GitHub Actions CI: lint + typecheck + test + build</t>
         </is>
       </c>
-      <c r="E86" s="7" t="inlineStr">
+      <c r="E88" s="7" t="inlineStr">
         <is>
           <t>As the team, we want CI to run lint/typecheck/test/build on every PR across all 3 packages, so that broken code can't merge to dev/main.
 AC1: CI SHALL run for backend, gateway, and frontend as separate jobs so a failure in one doesn't hide the others' results.
@@ -7115,74 +7266,74 @@
 AC3: A red CI run SHALL block merge per branch protection (07-github-workflow-git-conventions.md).</t>
         </is>
       </c>
-      <c r="F86" s="7" t="inlineStr">
+      <c r="F88" s="7" t="inlineStr">
         <is>
           <t>US-076</t>
         </is>
       </c>
-      <c r="G86" s="7" t="inlineStr">
+      <c r="G88" s="7" t="inlineStr">
         <is>
           <t>TK-84</t>
         </is>
       </c>
-      <c r="H86" s="7" t="inlineStr">
+      <c r="H88" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I86" s="7" t="inlineStr">
+      <c r="I88" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J86" s="7" t="n">
+      <c r="J88" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K86" s="7" t="inlineStr">
+      <c r="K88" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L86" s="7" t="inlineStr">
+      <c r="L88" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M86" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N86" s="7" t="inlineStr"/>
-      <c r="O86" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P86" s="7" t="inlineStr"/>
-    </row>
-    <row r="87" ht="60" customHeight="1">
-      <c r="A87" s="7" t="inlineStr">
+      <c r="M88" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N88" s="7" t="inlineStr"/>
+      <c r="O88" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P88" s="7" t="inlineStr"/>
+    </row>
+    <row r="89" ht="60" customHeight="1">
+      <c r="A89" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B87" s="7" t="inlineStr">
+      <c r="B89" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C87" s="7" t="inlineStr">
+      <c r="C89" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D87" s="7" t="inlineStr">
+      <c r="D89" s="7" t="inlineStr">
         <is>
           <t>GitHub Actions CD: build &amp; push images on merge</t>
         </is>
       </c>
-      <c r="E87" s="7" t="inlineStr">
+      <c r="E89" s="7" t="inlineStr">
         <is>
           <t>As Ops, I want images built and pushed on merge to main, so that a deployable artifact always exists for the current main branch state.
 AC1: The workflow SHALL build and tag images for backend/gateway/frontend on push to main.
@@ -7190,78 +7341,78 @@
 AC3: Image tags SHALL include the short commit SHA for traceability back to source.</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr">
+      <c r="F89" s="7" t="inlineStr">
         <is>
           <t>US-078</t>
         </is>
       </c>
-      <c r="G87" s="7" t="inlineStr">
+      <c r="G89" s="7" t="inlineStr">
         <is>
           <t>TK-86</t>
         </is>
       </c>
-      <c r="H87" s="7" t="inlineStr">
+      <c r="H89" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I87" s="7" t="inlineStr">
+      <c r="I89" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J87" s="7" t="n">
+      <c r="J89" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K87" s="7" t="inlineStr">
+      <c r="K89" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L87" s="7" t="inlineStr">
+      <c r="L89" s="7" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
-      <c r="M87" s="7" t="inlineStr">
+      <c r="M89" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N87" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="O87" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P87" s="7" t="inlineStr"/>
-    </row>
-    <row r="88" ht="60" customHeight="1">
-      <c r="A88" s="7" t="inlineStr">
+      <c r="N89" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="O89" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P89" s="7" t="inlineStr"/>
+    </row>
+    <row r="90" ht="60" customHeight="1">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C88" s="7" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D88" s="7" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>Deployment guide (clean-environment validated)</t>
         </is>
       </c>
-      <c r="E88" s="7" t="inlineStr">
+      <c r="E90" s="7" t="inlineStr">
         <is>
           <t>As the team, we want a deployment guide validated on a genuinely clean environment, so that Review 2/3 and the graders can stand the system up without tribal knowledge.
 AC1: The guide SHALL be followed literally on a fresh clone/VM by someone other than its author before being marked done.
@@ -7269,74 +7420,74 @@
 AC3: Any step that fails during validation SHALL be fixed in the guide, not worked around verbally.</t>
         </is>
       </c>
-      <c r="F88" s="7" t="inlineStr">
+      <c r="F90" s="7" t="inlineStr">
         <is>
           <t>US-080</t>
         </is>
       </c>
-      <c r="G88" s="7" t="inlineStr">
+      <c r="G90" s="7" t="inlineStr">
         <is>
           <t>TK-88</t>
         </is>
       </c>
-      <c r="H88" s="7" t="inlineStr">
+      <c r="H90" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I88" s="7" t="inlineStr">
+      <c r="I90" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J88" s="7" t="n">
+      <c r="J90" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K88" s="7" t="inlineStr">
+      <c r="K90" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L88" s="7" t="inlineStr">
+      <c r="L90" s="7" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
-      <c r="M88" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N88" s="7" t="inlineStr"/>
-      <c r="O88" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P88" s="7" t="inlineStr"/>
-    </row>
-    <row r="89" ht="60" customHeight="1">
-      <c r="A89" s="7" t="inlineStr">
+      <c r="M90" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N90" s="7" t="inlineStr"/>
+      <c r="O90" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P90" s="7" t="inlineStr"/>
+    </row>
+    <row r="91" ht="60" customHeight="1">
+      <c r="A91" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B89" s="7" t="inlineStr">
+      <c r="B91" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C89" s="7" t="inlineStr">
+      <c r="C91" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D89" s="7" t="inlineStr">
+      <c r="D91" s="7" t="inlineStr">
         <is>
           <t>Seed/demo data script</t>
         </is>
       </c>
-      <c r="E89" s="7" t="inlineStr">
+      <c r="E91" s="7" t="inlineStr">
         <is>
           <t>As the team, we want a seed script producing a runnable demonstration environment (sample devices, trips, one triggered incident), so that Review/Defense demos don't start from an empty database.
 AC1: The script SHALL populate a representative set of devices across all 7 lifecycle states.
@@ -7344,74 +7495,74 @@
 AC3: The script SHALL be idempotent, re-running it SHALL NOT duplicate seed data.</t>
         </is>
       </c>
-      <c r="F89" s="7" t="inlineStr">
+      <c r="F91" s="7" t="inlineStr">
         <is>
           <t>US-081</t>
         </is>
       </c>
-      <c r="G89" s="7" t="inlineStr">
+      <c r="G91" s="7" t="inlineStr">
         <is>
           <t>TK-89</t>
         </is>
       </c>
-      <c r="H89" s="7" t="inlineStr">
+      <c r="H91" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I89" s="7" t="inlineStr">
+      <c r="I91" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J89" s="7" t="n">
+      <c r="J91" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="K89" s="7" t="inlineStr">
+      <c r="K91" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L89" s="7" t="inlineStr">
+      <c r="L91" s="7" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
-      <c r="M89" s="7" t="inlineStr">
+      <c r="M91" s="7" t="inlineStr">
         <is>
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="N89" s="7" t="inlineStr"/>
-      <c r="O89" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P89" s="7" t="inlineStr"/>
-    </row>
-    <row r="90" ht="60" customHeight="1">
-      <c r="A90" s="7" t="inlineStr">
+      <c r="N91" s="7" t="inlineStr"/>
+      <c r="O91" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P91" s="7" t="inlineStr"/>
+    </row>
+    <row r="92" ht="60" customHeight="1">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B90" s="7" t="inlineStr">
+      <c r="B92" s="7" t="inlineStr">
         <is>
           <t>E7 - DevOps / CI-CD</t>
         </is>
       </c>
-      <c r="C90" s="7" t="inlineStr">
+      <c r="C92" s="7" t="inlineStr">
         <is>
           <t>X-DevOps</t>
         </is>
       </c>
-      <c r="D90" s="7" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Dockerfiles + docker-compose for all services</t>
         </is>
       </c>
-      <c r="E90" s="7" t="inlineStr">
+      <c r="E92" s="7" t="inlineStr">
         <is>
           <t>As a developer, I want Dockerfiles for backend/gateway/frontend plus a docker-compose stack (Postgres, Mosquitto), so that the whole platform runs with one command on any machine, satisfying the Deployability NFR.
 AC1: Each of backend/gateway/frontend SHALL have a working multi-stage Dockerfile.
@@ -7419,139 +7570,139 @@
 AC3: `docker compose up` SHALL bring up a working stack against a clean checkout with no manual steps beyond copying .env.example.</t>
         </is>
       </c>
-      <c r="F90" s="7" t="inlineStr">
+      <c r="F92" s="7" t="inlineStr">
         <is>
           <t>US-075</t>
         </is>
       </c>
-      <c r="G90" s="7" t="inlineStr">
+      <c r="G92" s="7" t="inlineStr">
         <is>
           <t>TK-83</t>
         </is>
       </c>
-      <c r="H90" s="7" t="inlineStr">
+      <c r="H92" s="7" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="I90" s="7" t="inlineStr">
+      <c r="I92" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J90" s="7" t="n">
+      <c r="J92" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K90" s="7" t="inlineStr">
+      <c r="K92" s="7" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="L90" s="7" t="inlineStr">
+      <c r="L92" s="7" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
-      <c r="M90" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N90" s="7" t="inlineStr">
+      <c r="M92" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N92" s="7" t="inlineStr">
         <is>
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="O90" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P90" s="7" t="inlineStr"/>
-    </row>
-    <row r="91" ht="60" customHeight="1">
-      <c r="A91" s="6" t="inlineStr">
+      <c r="O92" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P92" s="7" t="inlineStr"/>
+    </row>
+    <row r="93" ht="60" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C91" s="6" t="inlineStr"/>
-      <c r="D91" s="6" t="inlineStr">
+      <c r="C93" s="6" t="inlineStr"/>
+      <c r="D93" s="6" t="inlineStr">
         <is>
           <t>Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="E93" s="6" t="inlineStr">
         <is>
           <t>Added this session, homes the graded RQ1-RQ3 work that doesn't fit the other 7 template epics: the connectivity-loss experiment protocol/execution (RQ1/RQ2), the SOS-drill protocol/execution (RQ3), the end-to-end verification suite, and the evaluation report feeding Defense 1.
 Primary tables/entities: n/a (experiment protocol + evaluation report)</t>
         </is>
       </c>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="F93" s="6" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G93" s="6" t="inlineStr">
         <is>
           <t>TK-8</t>
         </is>
       </c>
-      <c r="H91" s="6" t="inlineStr"/>
-      <c r="I91" s="6" t="inlineStr"/>
-      <c r="J91" s="6" t="n">
+      <c r="H93" s="6" t="inlineStr"/>
+      <c r="I93" s="6" t="inlineStr"/>
+      <c r="J93" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="K91" s="6" t="inlineStr">
+      <c r="K93" s="6" t="inlineStr">
         <is>
           <t>Sprint 6 (cross-cutting research, not a Main Flow)</t>
         </is>
       </c>
-      <c r="L91" s="6" t="inlineStr"/>
-      <c r="M91" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N91" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="O91" s="6" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P91" s="6" t="inlineStr"/>
-    </row>
-    <row r="92" ht="60" customHeight="1">
-      <c r="A92" s="7" t="inlineStr">
+      <c r="L93" s="6" t="inlineStr"/>
+      <c r="M93" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N93" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="O93" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P93" s="6" t="inlineStr"/>
+    </row>
+    <row r="94" ht="60" customHeight="1">
+      <c r="A94" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B92" s="7" t="inlineStr">
+      <c r="B94" s="7" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="C94" s="7" t="inlineStr">
         <is>
           <t>X-Research</t>
         </is>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>Design RQ1/RQ2 connectivity-loss experiment protocol</t>
         </is>
       </c>
-      <c r="E92" s="7" t="inlineStr">
+      <c r="E94" s="7" t="inlineStr">
         <is>
           <t>As the team, we want the RQ1/RQ2 experiment protocol documented (connectivity-loss matrix, trial counts, measured variables) before running it, so that results are reproducible and defensible at Review 3/Defense 1.
 AC1: The protocol SHALL specify the connectivity-loss matrix exactly as registered: 0s/30s/2min/5min/10min/30min, 2 reconnection patterns, ≥20 trials/condition.
@@ -7559,74 +7710,74 @@
 AC3: The protocol SHALL be reviewed against 03-decisions-and-risk-register.md's risk mitigations before execution begins.</t>
         </is>
       </c>
-      <c r="F92" s="7" t="inlineStr">
+      <c r="F94" s="7" t="inlineStr">
         <is>
           <t>US-082</t>
         </is>
       </c>
-      <c r="G92" s="7" t="inlineStr">
+      <c r="G94" s="7" t="inlineStr">
         <is>
           <t>TK-90</t>
         </is>
       </c>
-      <c r="H92" s="7" t="inlineStr">
+      <c r="H94" s="7" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="I92" s="7" t="inlineStr">
+      <c r="I94" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J92" s="7" t="n">
+      <c r="J94" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K92" s="7" t="inlineStr">
+      <c r="K94" s="7" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="L92" s="7" t="inlineStr">
+      <c r="L94" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M92" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N92" s="7" t="inlineStr"/>
-      <c r="O92" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P92" s="7" t="inlineStr"/>
-    </row>
-    <row r="93" ht="60" customHeight="1">
-      <c r="A93" s="7" t="inlineStr">
+      <c r="M94" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N94" s="7" t="inlineStr"/>
+      <c r="O94" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P94" s="7" t="inlineStr"/>
+    </row>
+    <row r="95" ht="60" customHeight="1">
+      <c r="A95" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B93" s="7" t="inlineStr">
+      <c r="B95" s="7" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C95" s="7" t="inlineStr">
         <is>
           <t>X-Research</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D95" s="7" t="inlineStr">
         <is>
           <t>Design RQ3 SOS-drill experiment protocol</t>
         </is>
       </c>
-      <c r="E93" s="7" t="inlineStr">
+      <c r="E95" s="7" t="inlineStr">
         <is>
           <t>As the team, we want the RQ3 drill protocol documented (baseline vs. TrekLink condition, randomization, observer procedure), so that MTTA/MTTR/traceability comparisons are valid, not anecdotal.
 AC1: The protocol SHALL define the uncoordinated baseline exactly as registered (verbal/text acknowledgment, independent observer, hardware stopwatch, 0% traceability by definition).
@@ -7634,74 +7785,74 @@
 AC3: The protocol SHALL specify network-latency variation (LAN and 4G hotspot) as a controlled variable.</t>
         </is>
       </c>
-      <c r="F93" s="7" t="inlineStr">
+      <c r="F95" s="7" t="inlineStr">
         <is>
           <t>US-083</t>
         </is>
       </c>
-      <c r="G93" s="7" t="inlineStr">
+      <c r="G95" s="7" t="inlineStr">
         <is>
           <t>TK-91</t>
         </is>
       </c>
-      <c r="H93" s="7" t="inlineStr">
+      <c r="H95" s="7" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="I93" s="7" t="inlineStr">
+      <c r="I95" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J93" s="7" t="n">
+      <c r="J95" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K93" s="7" t="inlineStr">
+      <c r="K95" s="7" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="L93" s="7" t="inlineStr">
+      <c r="L95" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M93" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N93" s="7" t="inlineStr"/>
-      <c r="O93" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P93" s="7" t="inlineStr"/>
-    </row>
-    <row r="94" ht="60" customHeight="1">
-      <c r="A94" s="7" t="inlineStr">
+      <c r="M95" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N95" s="7" t="inlineStr"/>
+      <c r="O95" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P95" s="7" t="inlineStr"/>
+    </row>
+    <row r="96" ht="60" customHeight="1">
+      <c r="A96" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B94" s="7" t="inlineStr">
+      <c r="B96" s="7" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C94" s="7" t="inlineStr">
+      <c r="C96" s="7" t="inlineStr">
         <is>
           <t>X-Research</t>
         </is>
       </c>
-      <c r="D94" s="7" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
         <is>
           <t>Compile evaluation report</t>
         </is>
       </c>
-      <c r="E94" s="7" t="inlineStr">
+      <c r="E96" s="7" t="inlineStr">
         <is>
           <t>As the team, we want RQ1/RQ2/RQ3 results compiled into the evaluation report, so that Review 3 and Defense 1 have a single, complete, sourced document rather than scattered raw data.
 AC1: The report SHALL present RQ1/RQ2 results (delivery/loss/duplicate rate, latency, priority compliance) against the register's NFR targets.
@@ -7709,74 +7860,74 @@
 AC3: The report SHALL be cross-referenced from 00-project-context/02-roadmap-and-milestones.md's Review 3 checklist as a completed deliverable.</t>
         </is>
       </c>
-      <c r="F94" s="7" t="inlineStr">
+      <c r="F96" s="7" t="inlineStr">
         <is>
           <t>US-087</t>
         </is>
       </c>
-      <c r="G94" s="7" t="inlineStr">
+      <c r="G96" s="7" t="inlineStr">
         <is>
           <t>TK-95</t>
         </is>
       </c>
-      <c r="H94" s="7" t="inlineStr">
+      <c r="H96" s="7" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="I94" s="7" t="inlineStr">
+      <c r="I96" s="7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J94" s="7" t="n">
+      <c r="J96" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="K94" s="7" t="inlineStr">
+      <c r="K96" s="7" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="L94" s="7" t="inlineStr">
+      <c r="L96" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M94" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N94" s="7" t="inlineStr"/>
-      <c r="O94" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P94" s="7" t="inlineStr"/>
-    </row>
-    <row r="95" ht="60" customHeight="1">
-      <c r="A95" s="7" t="inlineStr">
+      <c r="M96" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N96" s="7" t="inlineStr"/>
+      <c r="O96" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P96" s="7" t="inlineStr"/>
+    </row>
+    <row r="97" ht="60" customHeight="1">
+      <c r="A97" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B95" s="7" t="inlineStr">
+      <c r="B97" s="7" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C95" s="7" t="inlineStr">
+      <c r="C97" s="7" t="inlineStr">
         <is>
           <t>X-Research</t>
         </is>
       </c>
-      <c r="D95" s="7" t="inlineStr">
+      <c r="D97" s="7" t="inlineStr">
         <is>
           <t>End-to-end integration test suite</t>
         </is>
       </c>
-      <c r="E95" s="7" t="inlineStr">
+      <c r="E97" s="7" t="inlineStr">
         <is>
           <t>As the team, we want an integration suite covering idempotency (10x replay), concurrency (20x simultaneous), RBAC validation, and audit-log completeness, so that the NFRs graded at Review 3 are continuously verified, not manually re-checked before the defense.
 AC1: The suite SHALL include the 10x-duplicate-eventId test (reuses US-052) and a 20-simultaneous-submission concurrency test with 0 duplicates asserted.
@@ -7784,74 +7935,74 @@
 AC3: The suite SHALL assert audit-log completeness: every FSM transition in a test run has a corresponding audit row.</t>
         </is>
       </c>
-      <c r="F95" s="7" t="inlineStr">
+      <c r="F97" s="7" t="inlineStr">
         <is>
           <t>US-086</t>
         </is>
       </c>
-      <c r="G95" s="7" t="inlineStr">
+      <c r="G97" s="7" t="inlineStr">
         <is>
           <t>TK-94</t>
         </is>
       </c>
-      <c r="H95" s="7" t="inlineStr">
+      <c r="H97" s="7" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="I95" s="7" t="inlineStr">
+      <c r="I97" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J95" s="7" t="n">
+      <c r="J97" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="K95" s="7" t="inlineStr">
+      <c r="K97" s="7" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="L95" s="7" t="inlineStr">
+      <c r="L97" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M95" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="N95" s="7" t="inlineStr"/>
-      <c r="O95" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P95" s="7" t="inlineStr"/>
-    </row>
-    <row r="96" ht="60" customHeight="1">
-      <c r="A96" s="7" t="inlineStr">
+      <c r="M97" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="N97" s="7" t="inlineStr"/>
+      <c r="O97" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P97" s="7" t="inlineStr"/>
+    </row>
+    <row r="98" ht="60" customHeight="1">
+      <c r="A98" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="B98" s="7" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C98" s="7" t="inlineStr">
         <is>
           <t>X-Research</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D98" s="7" t="inlineStr">
         <is>
           <t>Execute RQ1/RQ2 physical Gateway experiments</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr">
+      <c r="E98" s="7" t="inlineStr">
         <is>
           <t>As the team, we want to execute the RQ1/RQ2 protocol against 3-5 physical TrekLink devices and collect the metrics, so that the register's delivery-rate/latency/priority NFRs have empirical evidence, not an assumption.
 AC1: Physical devices SHALL be used for all mesh-to-gateway measurements; MQTT simulation may only supplement Gateway-to-Cloud load, never substitute for LoRa RF reliability claims.
@@ -7859,78 +8010,78 @@
 AC3: Raw results SHALL feed directly into US-087's evaluation report, not be re-summarized from memory afterward.</t>
         </is>
       </c>
-      <c r="F96" s="7" t="inlineStr">
+      <c r="F98" s="7" t="inlineStr">
         <is>
           <t>US-084</t>
         </is>
       </c>
-      <c r="G96" s="7" t="inlineStr">
+      <c r="G98" s="7" t="inlineStr">
         <is>
           <t>TK-92</t>
         </is>
       </c>
-      <c r="H96" s="7" t="inlineStr">
+      <c r="H98" s="7" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="I96" s="7" t="inlineStr">
+      <c r="I98" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J96" s="7" t="n">
+      <c r="J98" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="K96" s="7" t="inlineStr">
+      <c r="K98" s="7" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="L96" s="7" t="inlineStr">
+      <c r="L98" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M96" s="7" t="inlineStr">
+      <c r="M98" s="7" t="inlineStr">
         <is>
           <t>Lâm Phi Long</t>
         </is>
       </c>
-      <c r="N96" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="O96" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P96" s="7" t="inlineStr"/>
-    </row>
-    <row r="97" ht="60" customHeight="1">
-      <c r="A97" s="7" t="inlineStr">
+      <c r="N98" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="O98" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P98" s="7" t="inlineStr"/>
+    </row>
+    <row r="99" ht="60" customHeight="1">
+      <c r="A99" s="7" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B97" s="7" t="inlineStr">
+      <c r="B99" s="7" t="inlineStr">
         <is>
           <t>E8 - Research &amp; Experimental Evaluation</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="C99" s="7" t="inlineStr">
         <is>
           <t>X-Research</t>
         </is>
       </c>
-      <c r="D97" s="7" t="inlineStr">
+      <c r="D99" s="7" t="inlineStr">
         <is>
           <t>Execute RQ3 randomized SOS drills</t>
         </is>
       </c>
-      <c r="E97" s="7" t="inlineStr">
+      <c r="E99" s="7" t="inlineStr">
         <is>
           <t>As the team, we want to execute the RQ3 drill protocol (baseline + TrekLink condition) and collect MTTA/MTTR/traceability/completion-rate data, so that the SOS-to-Incident pipeline's improvement over the status quo is measured, not assumed.
 AC1: Drills SHALL run per the protocol from US-084 with an independent observer and randomized trigger timing.
@@ -7938,72 +8089,72 @@
 AC3: A reduction in MTTA SHALL NOT be assumed in advance, outcomes are reported as measured, per the register's own stated caution.</t>
         </is>
       </c>
-      <c r="F97" s="7" t="inlineStr">
+      <c r="F99" s="7" t="inlineStr">
         <is>
           <t>US-085</t>
         </is>
       </c>
-      <c r="G97" s="7" t="inlineStr">
+      <c r="G99" s="7" t="inlineStr">
         <is>
           <t>TK-93</t>
         </is>
       </c>
-      <c r="H97" s="7" t="inlineStr">
+      <c r="H99" s="7" t="inlineStr">
         <is>
           <t>E8</t>
         </is>
       </c>
-      <c r="I97" s="7" t="inlineStr">
+      <c r="I99" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J97" s="7" t="n">
+      <c r="J99" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="K97" s="7" t="inlineStr">
+      <c r="K99" s="7" t="inlineStr">
         <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="L97" s="7" t="inlineStr">
+      <c r="L99" s="7" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="M97" s="7" t="inlineStr">
+      <c r="M99" s="7" t="inlineStr">
         <is>
           <t>Nguyễn Bá Tân</t>
         </is>
       </c>
-      <c r="N97" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="O97" s="7" t="inlineStr">
-        <is>
-          <t>Đỗ Đăng Khoa</t>
-        </is>
-      </c>
-      <c r="P97" s="7" t="inlineStr"/>
+      <c r="N99" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="O99" s="7" t="inlineStr">
+        <is>
+          <t>Đỗ Đăng Khoa</t>
+        </is>
+      </c>
+      <c r="P99" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <dataValidations count="5">
-    <dataValidation sqref="A2:A97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A2:A99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Epic,Story"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"E1 - Identity &amp; RBAC,E2 - Device Fleet &amp; Maintenance,E3 - Trip &amp; Rental Management,E4 - Gateway &amp; Offline Sync,E5 - Real-Time Monitoring &amp; SOS Incidents,E6 - Billing &amp; Reporting,E7 - DevOps / CI-CD,E8 - Research &amp; Experimental Evaluation"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,5,8,13"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Backlog,Ready,In Progress,In Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8245,10 +8396,10 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
@@ -8477,10 +8628,10 @@
       </c>
       <c r="C10" s="8" t="inlineStr"/>
       <c r="D10" s="8" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>365</v>
+        <v>391</v>
       </c>
       <c r="F10" s="8" t="inlineStr"/>
       <c r="G10" s="8" t="inlineStr"/>
@@ -8577,10 +8728,10 @@
         </is>
       </c>
       <c r="D2" s="7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="F2" s="7" t="n">
         <v>6</v>
@@ -8590,7 +8741,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>26.6%</t>
+          <t>31.5%</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -8629,7 +8780,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -8668,7 +8819,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.0%</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -8707,7 +8858,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>11.8%</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -8746,7 +8897,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -8764,10 +8915,10 @@
       <c r="B7" s="8" t="inlineStr"/>
       <c r="C7" s="8" t="inlineStr"/>
       <c r="D7" s="8" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>365</v>
+        <v>391</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>20</v>

</xml_diff>

<commit_message>
docs: file the map sovereignty evidence and pull auth into Sprint 2
D-012 and 07 record that the Goong and OpenStreetMap screenshots are filed in capstone/Documents/evidence/map-sovereignty; TC-24 passes for Goong. The backlog pulls the auth stories into Sprint 2 so MF-01 can finish before Review 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -933,7 +933,7 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -1392,12 +1392,12 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: file the map sovereignty evidence and pull auth into Sprint 2 (#32)
* docs: file the map sovereignty evidence and pull auth into Sprint 2

D-012 and 07 record that the Goong and OpenStreetMap screenshots are filed in capstone/Documents/evidence/map-sovereignty; TC-24 passes for Goong. The backlog pulls the auth stories into Sprint 2 so MF-01 can finish before Review 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* docs(conventions): graded documents never cite internal records

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* docs: rebuild developer handbook PDF [skip ci]

---------

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -933,7 +933,7 @@
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -1392,12 +1392,12 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 2</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: align backlog Jira keys with the keys Jira issued (D-029)
The first jira_sync.py run found TK-1 to TK-5 already in the project, so the epics became
TK-6 to TK-13 and the stories TK-14 to TK-103. The key bases move to 6 and 14 and the
backlog, xlsx and chapter 10 example are regenerated to match. jira_sync.py now rejects a
non-numeric JIRA_BOARD_ID before creating any card; the first run crashed on it after the
cards were made, so no sprints were created.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -848,7 +848,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>TK-1</t>
+          <t>TK-6</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>TK-14</t>
+          <t>TK-19</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>TK-10</t>
+          <t>TK-15</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>TK-11</t>
+          <t>TK-16</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>TK-12</t>
+          <t>TK-17</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>TK-15</t>
+          <t>TK-20</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>TK-18</t>
+          <t>TK-23</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>TK-9</t>
+          <t>TK-14</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>TK-13</t>
+          <t>TK-18</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>TK-16</t>
+          <t>TK-21</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>TK-17</t>
+          <t>TK-22</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>TK-2</t>
+          <t>TK-7</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>TK-24</t>
+          <t>TK-29</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>TK-28</t>
+          <t>TK-33</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>TK-29</t>
+          <t>TK-34</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>TK-19</t>
+          <t>TK-24</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>TK-20</t>
+          <t>TK-25</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>TK-23</t>
+          <t>TK-28</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>TK-26</t>
+          <t>TK-31</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>TK-27</t>
+          <t>TK-32</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>TK-30</t>
+          <t>TK-35</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>TK-22</t>
+          <t>TK-27</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>TK-25</t>
+          <t>TK-30</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>TK-21</t>
+          <t>TK-26</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>TK-3</t>
+          <t>TK-8</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>TK-32</t>
+          <t>TK-37</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>TK-39</t>
+          <t>TK-44</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>TK-48</t>
+          <t>TK-53</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>TK-31</t>
+          <t>TK-36</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>TK-35</t>
+          <t>TK-40</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>TK-37</t>
+          <t>TK-42</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>TK-41</t>
+          <t>TK-46</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>TK-43</t>
+          <t>TK-48</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>TK-44</t>
+          <t>TK-49</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>TK-45</t>
+          <t>TK-50</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>TK-47</t>
+          <t>TK-52</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>TK-33</t>
+          <t>TK-38</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>TK-34</t>
+          <t>TK-39</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>TK-36</t>
+          <t>TK-41</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>TK-38</t>
+          <t>TK-43</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>TK-40</t>
+          <t>TK-45</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>TK-42</t>
+          <t>TK-47</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>TK-46</t>
+          <t>TK-51</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>TK-4</t>
+          <t>TK-9</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>TK-50</t>
+          <t>TK-55</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>TK-53</t>
+          <t>TK-58</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>TK-57</t>
+          <t>TK-62</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>TK-60</t>
+          <t>TK-65</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>TK-51</t>
+          <t>TK-56</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>TK-52</t>
+          <t>TK-57</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>TK-54</t>
+          <t>TK-59</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>TK-55</t>
+          <t>TK-60</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>TK-59</t>
+          <t>TK-64</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>TK-49</t>
+          <t>TK-54</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>TK-56</t>
+          <t>TK-61</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>TK-58</t>
+          <t>TK-63</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>TK-97</t>
+          <t>TK-102</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>TK-98</t>
+          <t>TK-103</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>TK-5</t>
+          <t>TK-10</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -5267,7 +5267,7 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>TK-64</t>
+          <t>TK-69</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>TK-67</t>
+          <t>TK-72</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>TK-68</t>
+          <t>TK-73</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>TK-69</t>
+          <t>TK-74</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>TK-70</t>
+          <t>TK-75</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>TK-72</t>
+          <t>TK-77</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>TK-73</t>
+          <t>TK-78</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>TK-74</t>
+          <t>TK-79</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>TK-61</t>
+          <t>TK-66</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>TK-65</t>
+          <t>TK-70</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>TK-66</t>
+          <t>TK-71</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>TK-71</t>
+          <t>TK-76</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>TK-96</t>
+          <t>TK-101</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>TK-62</t>
+          <t>TK-67</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>TK-63</t>
+          <t>TK-68</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>TK-6</t>
+          <t>TK-11</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>TK-78</t>
+          <t>TK-83</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>TK-81</t>
+          <t>TK-86</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>TK-82</t>
+          <t>TK-87</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>TK-77</t>
+          <t>TK-82</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>TK-79</t>
+          <t>TK-84</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>TK-80</t>
+          <t>TK-85</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>TK-75</t>
+          <t>TK-80</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>TK-76</t>
+          <t>TK-81</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>TK-7</t>
+          <t>TK-12</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
@@ -7123,7 +7123,7 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>TK-85</t>
+          <t>TK-90</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>TK-87</t>
+          <t>TK-92</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>TK-84</t>
+          <t>TK-89</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>TK-86</t>
+          <t>TK-91</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>TK-88</t>
+          <t>TK-93</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
@@ -7502,7 +7502,7 @@
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>TK-89</t>
+          <t>TK-94</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>TK-83</t>
+          <t>TK-88</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>TK-8</t>
+          <t>TK-13</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>TK-90</t>
+          <t>TK-95</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
@@ -7792,7 +7792,7 @@
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>TK-91</t>
+          <t>TK-96</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>TK-95</t>
+          <t>TK-100</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>TK-94</t>
+          <t>TK-99</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
@@ -8017,7 +8017,7 @@
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>TK-92</t>
+          <t>TK-97</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>TK-93</t>
+          <t>TK-98</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: align backlog Jira keys with the keys Jira issued (D-029) (#33)
* docs: align backlog Jira keys with the keys Jira issued (D-029)

The first jira_sync.py run found TK-1 to TK-5 already in the project, so the epics became
TK-6 to TK-13 and the stories TK-14 to TK-103. The key bases move to 6 and 14 and the
backlog, xlsx and chapter 10 example are regenerated to match. jira_sync.py now rejects a
non-numeric JIRA_BOARD_ID before creating any card; the first run crashed on it after the
cards were made, so no sprints were created.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* docs: rebuild developer handbook PDF [skip ci]

---------

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -848,7 +848,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>TK-1</t>
+          <t>TK-6</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>TK-14</t>
+          <t>TK-19</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>TK-10</t>
+          <t>TK-15</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>TK-11</t>
+          <t>TK-16</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>TK-12</t>
+          <t>TK-17</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>TK-15</t>
+          <t>TK-20</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>TK-18</t>
+          <t>TK-23</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>TK-9</t>
+          <t>TK-14</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>TK-13</t>
+          <t>TK-18</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>TK-16</t>
+          <t>TK-21</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>TK-17</t>
+          <t>TK-22</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>TK-2</t>
+          <t>TK-7</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>TK-24</t>
+          <t>TK-29</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>TK-28</t>
+          <t>TK-33</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>TK-29</t>
+          <t>TK-34</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>TK-19</t>
+          <t>TK-24</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>TK-20</t>
+          <t>TK-25</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>TK-23</t>
+          <t>TK-28</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>TK-26</t>
+          <t>TK-31</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>TK-27</t>
+          <t>TK-32</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>TK-30</t>
+          <t>TK-35</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>TK-22</t>
+          <t>TK-27</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>TK-25</t>
+          <t>TK-30</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>TK-21</t>
+          <t>TK-26</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>TK-3</t>
+          <t>TK-8</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>TK-32</t>
+          <t>TK-37</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>TK-39</t>
+          <t>TK-44</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>TK-48</t>
+          <t>TK-53</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>TK-31</t>
+          <t>TK-36</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>TK-35</t>
+          <t>TK-40</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>TK-37</t>
+          <t>TK-42</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>TK-41</t>
+          <t>TK-46</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>TK-43</t>
+          <t>TK-48</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>TK-44</t>
+          <t>TK-49</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>TK-45</t>
+          <t>TK-50</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>TK-47</t>
+          <t>TK-52</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>TK-33</t>
+          <t>TK-38</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>TK-34</t>
+          <t>TK-39</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>TK-36</t>
+          <t>TK-41</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
@@ -3774,7 +3774,7 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>TK-38</t>
+          <t>TK-43</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>TK-40</t>
+          <t>TK-45</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>TK-42</t>
+          <t>TK-47</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>TK-46</t>
+          <t>TK-51</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>TK-4</t>
+          <t>TK-9</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>TK-50</t>
+          <t>TK-55</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>TK-53</t>
+          <t>TK-58</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>TK-57</t>
+          <t>TK-62</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>TK-60</t>
+          <t>TK-65</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>TK-51</t>
+          <t>TK-56</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>TK-52</t>
+          <t>TK-57</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>TK-54</t>
+          <t>TK-59</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>TK-55</t>
+          <t>TK-60</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>TK-59</t>
+          <t>TK-64</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>TK-49</t>
+          <t>TK-54</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>TK-56</t>
+          <t>TK-61</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>TK-58</t>
+          <t>TK-63</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>TK-97</t>
+          <t>TK-102</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
@@ -5131,7 +5131,7 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>TK-98</t>
+          <t>TK-103</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>TK-5</t>
+          <t>TK-10</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr"/>
@@ -5267,7 +5267,7 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>TK-64</t>
+          <t>TK-69</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>TK-67</t>
+          <t>TK-72</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>TK-68</t>
+          <t>TK-73</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>TK-69</t>
+          <t>TK-74</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>TK-70</t>
+          <t>TK-75</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>TK-72</t>
+          <t>TK-77</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>TK-73</t>
+          <t>TK-78</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>TK-74</t>
+          <t>TK-79</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>TK-61</t>
+          <t>TK-66</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>TK-65</t>
+          <t>TK-70</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>TK-66</t>
+          <t>TK-71</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>TK-71</t>
+          <t>TK-76</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>TK-96</t>
+          <t>TK-101</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>TK-62</t>
+          <t>TK-67</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>TK-63</t>
+          <t>TK-68</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>TK-6</t>
+          <t>TK-11</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr"/>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>TK-78</t>
+          <t>TK-83</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>TK-81</t>
+          <t>TK-86</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>TK-82</t>
+          <t>TK-87</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>TK-77</t>
+          <t>TK-82</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>TK-79</t>
+          <t>TK-84</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
@@ -6837,7 +6837,7 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>TK-80</t>
+          <t>TK-85</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>TK-75</t>
+          <t>TK-80</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>TK-76</t>
+          <t>TK-81</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>TK-7</t>
+          <t>TK-12</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr"/>
@@ -7123,7 +7123,7 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>TK-85</t>
+          <t>TK-90</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>TK-87</t>
+          <t>TK-92</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>TK-84</t>
+          <t>TK-89</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>TK-86</t>
+          <t>TK-91</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>TK-88</t>
+          <t>TK-93</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
@@ -7502,7 +7502,7 @@
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>TK-89</t>
+          <t>TK-94</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>TK-83</t>
+          <t>TK-88</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>TK-8</t>
+          <t>TK-13</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr"/>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>TK-90</t>
+          <t>TK-95</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
@@ -7792,7 +7792,7 @@
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>TK-91</t>
+          <t>TK-96</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
@@ -7867,7 +7867,7 @@
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>TK-95</t>
+          <t>TK-100</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>TK-94</t>
+          <t>TK-99</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
@@ -8017,7 +8017,7 @@
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>TK-92</t>
+          <t>TK-97</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>TK-93</t>
+          <t>TK-98</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: record D-031, the map reverts to Leaflet over OpenStreetMap
The supervisor accepts OpenStreetMap for the course. D-031 supersedes D-012:
Leaflet renders OpenStreetMap tiles, Goong Maps stays dormant in
configuration, and a mandatory overlay labels Hoang Sa and Truong Sa in
Vietnamese. R11 is reopened as an accepted risk within educational scope.

Conventions, charter, roadmap, Main Flows, requirements foundation, US-055
and the canonical AGENTS.md follow. The handbook PDF is rebuilt (D-025).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -6304,15 +6304,16 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Live operational map (MapLibre GL + Goong Maps)</t>
+          <t>Live operational map (Leaflet + OpenStreetMap)</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
           <t>As Staff/Admin/Guide, I want a live map showing active trip positions, so that I have field situational awareness without polling manually.
 AC1: The map SHALL render device/trip markers colored by status per Pattern B (06-frontend-conventions.md §4).
-AC2: Position updates SHALL arrive via the shared WebSocket channel (US-053), not polling.
-AC3: The map SHALL be the LiveMapWidget consumed by both the Staff dashboard and the Guide's own trip view (US-038).</t>
+AC2: The map SHALL carry the Vietnamese sovereignty overlay over Hoàng Sa and Trường Sa (D-031).
+AC3: Position updates SHALL arrive via the shared WebSocket channel (US-053), not polling.
+AC4: The map SHALL be the LiveMapWidget consumed by both the Staff dashboard and the Guide's own trip view (US-038).</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">

</xml_diff>

<commit_message>
docs: close the D-056 follow-ups
Confirm D-056 as the leader's ruling, word task 2.3 as the single
exception, add the Review 2 fallback for tasks 1.1 and 2.1 and the
HoangTK acknowledgement. Give the monitoring lane to LongNN in
build_backlog.py with HoangTK as secondary, regenerate the backlog,
and align the chapter 11 lane table with roadmap section 5.1.

Checksum: 0e3222e26e331246d8b0f3261651222e9dffeda93a6907972ad761f585c0193a
</commit_message>
<xml_diff>
--- a/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
+++ b/_docs/00-project-context/User_Story_Agile_TrekLink.xlsx
@@ -3083,7 +3083,7 @@
 FR-EVT-05: IF a payload cannot be decoded, THEN the system SHALL log it raw, count it, drop it and continue without blocking the queue head.
 FR-EVT-08: The system SHALL order events by queue sequence and priority, never by wall-clock comparison across hosts, and SHALL treat a device `rx_time` of 0 as unknown.
 FR-EVT-09: WHEN a text event is decoded, the system SHALL test the `SOS - FALL DETECTED` prefix before the `SOS - ` prefix and SHALL classify both as SOS.
-FR-EVT-10: The system SHALL accept events from the stock Meshtastic MQTT topics `&lt;root&gt;/2/json/...` and `&lt;root&gt;/2/e/...` through ingress adapters that produce one canonical event envelope.
+FR-EVT-10: The system SHALL accept events from the stock Meshtastic MQTT JSON topic `&lt;root&gt;/2/json/...` through an ingress adapter that produces one canonical event envelope; the protobuf topic `&lt;root&gt;/2/e/...` stays permitted by the broker and is not ingested.
 FR-EVT-11: The system SHALL write one append-only synchronization audit row per ingestion attempt, recording acceptance or duplicate rejection.
 FR-EVT-14: WHEN an Org Manager creates a Field Station credential, the system SHALL show it once, store only its hash, bind it to the organization, and accept MQTT publishes under it only for devices the organization rents, or returned within the configured late-upload grace period; WHEN the Manager, TrekLink Staff or an Admin revokes it, the broker SHALL refuse it from the next connection.
 FR-EVT-15: WHEN a field event is ingested, the system SHALL record its server receipt time and SHALL derive its occurrence time, recording the source used: the Field Station's capture time corrected by the clock offset the station reports at each sync; otherwise the device `rx_time` when it is non-zero and within the configured plausibility window before receipt; otherwise the receipt time. Occurrence time SHALL be used for attribution only, never for ordering events across hosts.
@@ -4005,7 +4005,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>HoangTK</t>
+          <t>LongNN</t>
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>HoangTK</t>
+          <t>LongNN</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -4129,7 +4129,7 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>HoangTK</t>
+          <t>LongNN</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
@@ -6561,17 +6561,17 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>incidents, monitoring</t>
+          <t>incidents</t>
         </is>
       </c>
     </row>
@@ -6587,13 +6587,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>

</xml_diff>